<commit_message>
Correct timezone description of IANA database
</commit_message>
<xml_diff>
--- a/models/all-to-all-mapping.xlsx
+++ b/models/all-to-all-mapping.xlsx
@@ -19,19 +19,19 @@
 <comments xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision">
   <authors>
     <author/>
-    <author>tc={0c56af75-6606-4500-b0e0-efb6e4ee024c}</author>
-    <author>tc={14a075e4-3e63-45dd-873b-d4b67be1f443}</author>
-    <author>tc={194dfa0d-f86e-48fa-aa6a-8fca58e121aa}</author>
-    <author>tc={1ce51903-2067-4d3a-ac25-0103b7cbba14}</author>
-    <author>tc={711133ba-b785-4ddc-91ee-65c1a80128d2}</author>
-    <author>tc={797089d9-9fef-4104-a3bd-35403993da1d}</author>
-    <author>tc={799f37c3-35ee-48b3-8d2f-783c9ecca11b}</author>
-    <author>tc={8fbcdf78-ef70-4737-aa2f-226525291599}</author>
-    <author>tc={c2df04c0-8527-437b-935e-02e7db7acb5f}</author>
-    <author>tc={c93ec52d-3811-4e8e-8987-a0e04d67fed5}</author>
-    <author>tc={e76141e3-8a70-4937-9879-b614dd0e3767}</author>
-    <author>tc={eb3bd140-efca-406a-8d17-195ddc05469c}</author>
-    <author>tc={efabe969-7dca-426e-acf9-b3c8261a837f}</author>
+    <author>tc={34973966-2beb-456a-b13f-8d4c654fcc70}</author>
+    <author>tc={419191be-88a2-4ebb-a9d0-45b001253b72}</author>
+    <author>tc={492be683-d186-43f6-8398-65826dbb9411}</author>
+    <author>tc={4e41cf75-544b-4e1e-a9ca-ddfa81e299ad}</author>
+    <author>tc={4f1e0add-0afa-4f26-a2f2-76800d1c42cc}</author>
+    <author>tc={5958f09c-2156-4518-8c68-755ee955ef16}</author>
+    <author>tc={5fbae45b-a0ee-4e46-816c-a61f09720000}</author>
+    <author>tc={655fe435-7a29-4e9b-a1f1-627dbaa873fa}</author>
+    <author>tc={7513edb4-21ae-4d7f-a667-8b566e125b23}</author>
+    <author>tc={86067411-4f64-4dea-bb8c-484eb0624e97}</author>
+    <author>tc={9b74a778-7338-4d64-b624-90b4eaee3552}</author>
+    <author>tc={b8c87507-4a8d-4067-bb0d-ad3535e9bfd0}</author>
+    <author>tc={f52a97ab-1ac4-42b5-a810-0c62e3171378}</author>
   </authors>
   <commentList>
     <comment authorId="0" ref="R18">
@@ -69,7 +69,35 @@
         <t xml:space="preserve">inLanguage is recommended in Bioschemas and we don't yet serialize it</t>
       </text>
     </comment>
-    <comment authorId="1" xr:uid="{0c56af75-6606-4500-b0e0-efb6e4ee024c}" ref="J47">
+    <comment authorId="1" xr:uid="{34973966-2beb-456a-b13f-8d4c654fcc70}" ref="N30">
+      <text>
+        <t xml:space="preserve">[Threaded comment]
+ Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+	Is this the best way to record timezone?
+</t>
+      </text>
+    </comment>
+    <comment authorId="2" xr:uid="{419191be-88a2-4ebb-a9d0-45b001253b72}" ref="J16">
+      <text>
+        <t xml:space="preserve">[Threaded comment]
+ Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+	EOSC 2024 schema has 'Expertise Level'. TeSS has 'Competency Level' and the Bioschemas 'educationalLevel' property, limited to the values of 'Beginner', 'Intermediate', 'Advanced'. 
+This might be better represented as two separate properties. Consider Terms4FAIRskills vocabulary for one of these.
+</t>
+      </text>
+    </comment>
+    <comment authorId="3" xr:uid="{492be683-d186-43f6-8398-65826dbb9411}" ref="L35">
+      <text>
+        <t xml:space="preserve">[Threaded comment]
+ Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+	Could use 2 or 3 character ISO 3166 country code
+</t>
+      </text>
+    </comment>
+    <comment authorId="4" xr:uid="{4e41cf75-544b-4e1e-a9ca-ddfa81e299ad}" ref="J47">
       <text>
         <t xml:space="preserve">[Threaded comment]
  Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -78,7 +106,7 @@
 </t>
       </text>
     </comment>
-    <comment authorId="2" xr:uid="{14a075e4-3e63-45dd-873b-d4b67be1f443}" ref="J7">
+    <comment authorId="5" xr:uid="{4f1e0add-0afa-4f26-a2f2-76800d1c42cc}" ref="J7">
       <text>
         <t xml:space="preserve">[Threaded comment]
  Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -89,7 +117,26 @@
 </t>
       </text>
     </comment>
-    <comment authorId="3" xr:uid="{194dfa0d-f86e-48fa-aa6a-8fca58e121aa}" ref="K32">
+    <comment authorId="6" xr:uid="{5958f09c-2156-4518-8c68-755ee955ef16}" ref="J12">
+      <text>
+        <t xml:space="preserve">[Threaded comment]
+ Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+	Base TeSS does not mandate license, too many materials would be rejected. 
+Also, TeSS events do not have license (it is not in the Bioschemas profile).
+</t>
+      </text>
+    </comment>
+    <comment authorId="7" xr:uid="{5fbae45b-a0ee-4e46-816c-a61f09720000}" ref="L7">
+      <text>
+        <t xml:space="preserve">[Threaded comment]
+ Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+	TeSS currently supports two "levels" of material contribution: 'author' and 'contributor'. For events, this changes to 'Organizer' which may be a person or an organization. Our workshop proposed extending this beyond author and contributor, to an existing CV. It is not clear to me from the notes which is suitable. (We also propose including ORCID for 'organizer' of an event'.)
+</t>
+      </text>
+    </comment>
+    <comment authorId="8" xr:uid="{655fe435-7a29-4e9b-a1f1-627dbaa873fa}" ref="K32">
       <text>
         <t xml:space="preserve">[Threaded comment]
  Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -98,7 +145,25 @@
 </t>
       </text>
     </comment>
-    <comment authorId="4" xr:uid="{1ce51903-2067-4d3a-ac25-0103b7cbba14}" ref="L42">
+    <comment authorId="9" xr:uid="{7513edb4-21ae-4d7f-a667-8b566e125b23}" ref="N7">
+      <text>
+        <t xml:space="preserve">[Threaded comment]
+ Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+	TODO: Role
+</t>
+      </text>
+    </comment>
+    <comment authorId="10" xr:uid="{86067411-4f64-4dea-bb8c-484eb0624e97}" ref="N18">
+      <text>
+        <t xml:space="preserve">[Threaded comment]
+ Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+	Add to Bioschemas
+</t>
+      </text>
+    </comment>
+    <comment authorId="11" xr:uid="{9b74a778-7338-4d64-b624-90b4eaee3552}" ref="L42">
       <text>
         <t xml:space="preserve">[Threaded comment]
  Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -108,53 +173,7 @@
 </t>
       </text>
     </comment>
-    <comment authorId="5" xr:uid="{711133ba-b785-4ddc-91ee-65c1a80128d2}" ref="N18">
-      <text>
-        <t xml:space="preserve">[Threaded comment]
- Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
-	Add to Bioschemas
-</t>
-      </text>
-    </comment>
-    <comment authorId="6" xr:uid="{797089d9-9fef-4104-a3bd-35403993da1d}" ref="L35">
-      <text>
-        <t xml:space="preserve">[Threaded comment]
- Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
-	Could use 2 or 3 character ISO 3166 country code
-</t>
-      </text>
-    </comment>
-    <comment authorId="7" xr:uid="{799f37c3-35ee-48b3-8d2f-783c9ecca11b}" ref="N7">
-      <text>
-        <t xml:space="preserve">[Threaded comment]
- Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
-	TODO: Role
-</t>
-      </text>
-    </comment>
-    <comment authorId="8" xr:uid="{8fbcdf78-ef70-4737-aa2f-226525291599}" ref="L1">
-      <text>
-        <t xml:space="preserve">[Threaded comment]
- Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
-	Still to define: controlled vocabularies
-</t>
-      </text>
-    </comment>
-    <comment authorId="9" xr:uid="{c2df04c0-8527-437b-935e-02e7db7acb5f}" ref="J16">
-      <text>
-        <t xml:space="preserve">[Threaded comment]
- Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
-	EOSC 2024 schema has 'Expertise Level'. TeSS has 'Competency Level' and the Bioschemas 'educationalLevel' property, limited to the values of 'Beginner', 'Intermediate', 'Advanced'. 
-This might be better represented as two separate properties. Consider Terms4FAIRskills vocabulary for one of these.
-</t>
-      </text>
-    </comment>
-    <comment authorId="10" xr:uid="{c93ec52d-3811-4e8e-8987-a0e04d67fed5}" ref="N42">
+    <comment authorId="12" xr:uid="{b8c87507-4a8d-4067-bb0d-ad3535e9bfd0}" ref="N42">
       <text>
         <t xml:space="preserve">[Threaded comment]
  Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -163,31 +182,12 @@
 </t>
       </text>
     </comment>
-    <comment authorId="11" xr:uid="{e76141e3-8a70-4937-9879-b614dd0e3767}" ref="L7">
+    <comment authorId="13" xr:uid="{f52a97ab-1ac4-42b5-a810-0c62e3171378}" ref="L1">
       <text>
         <t xml:space="preserve">[Threaded comment]
  Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
-	TeSS currently supports two "levels" of material contribution: 'author' and 'contributor'. For events, this changes to 'Organizer' which may be a person or an organization. Our workshop proposed extending this beyond author and contributor, to an existing CV. It is not clear to me from the notes which is suitable. (We also propose including ORCID for 'organizer' of an event'.)
-</t>
-      </text>
-    </comment>
-    <comment authorId="12" xr:uid="{eb3bd140-efca-406a-8d17-195ddc05469c}" ref="J12">
-      <text>
-        <t xml:space="preserve">[Threaded comment]
- Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
-	Base TeSS does not mandate license, too many materials would be rejected. 
-Also, TeSS events do not have license (it is not in the Bioschemas profile).
-</t>
-      </text>
-    </comment>
-    <comment authorId="13" xr:uid="{efabe969-7dca-426e-acf9-b3c8261a837f}" ref="N30">
-      <text>
-        <t xml:space="preserve">[Threaded comment]
- Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
-	Is this the best way to record timezone?
+	Still to define: controlled vocabularies
 </t>
       </text>
     </comment>
@@ -1024,7 +1024,7 @@
     <t>Timezone</t>
   </si>
   <si>
-    <t>IANA RFC 6557</t>
+    <t>IANA</t>
   </si>
   <si>
     <t>Duration</t>
@@ -1733,7 +1733,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="25">
+  <fonts count="26">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -1783,6 +1783,11 @@
     <font>
       <u/>
       <color rgb="FF0000FF"/>
+    </font>
+    <font>
+      <u/>
+      <color rgb="FF0000FF"/>
+      <name val="Arial"/>
     </font>
     <font>
       <u/>
@@ -2189,7 +2194,7 @@
     <xf borderId="1" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment vertical="top"/>
     </xf>
-    <xf borderId="1" fillId="7" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="1" fillId="7" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0" vertical="top"/>
     </xf>
     <xf borderId="0" fillId="7" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
@@ -2201,7 +2206,7 @@
     <xf borderId="0" fillId="7" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" vertical="top"/>
     </xf>
-    <xf borderId="1" fillId="7" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="1" fillId="7" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="top" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="7" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
@@ -2210,10 +2215,10 @@
     <xf borderId="1" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="top" wrapText="0"/>
     </xf>
-    <xf borderId="1" fillId="7" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="1" fillId="7" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="top" wrapText="0"/>
     </xf>
-    <xf borderId="1" fillId="7" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="1" fillId="7" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="top" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
@@ -2222,7 +2227,7 @@
     <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment shrinkToFit="0" wrapText="0"/>
     </xf>
-    <xf borderId="0" fillId="7" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="7" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="top" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="11" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
@@ -2232,11 +2237,11 @@
     <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="14" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="14" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="15" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf borderId="0" fillId="0" fontId="16" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="6" fontId="3" numFmtId="0" xfId="0" applyFont="1"/>
@@ -2247,10 +2252,10 @@
     <xf borderId="0" fillId="9" fontId="3" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="0" fillId="13" fontId="3" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="0" fillId="10" fontId="3" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="16" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="17" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="17" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="18" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
     <xf borderId="1" fillId="7" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
@@ -2263,41 +2268,41 @@
     <xf borderId="1" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="18" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="1" fillId="0" fontId="19" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="3" fillId="5" fontId="19" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="3" fillId="5" fontId="20" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0" vertical="top"/>
     </xf>
-    <xf borderId="3" fillId="2" fontId="20" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="3" fillId="2" fontId="21" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0" vertical="top"/>
     </xf>
-    <xf borderId="3" fillId="7" fontId="19" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="3" fillId="7" fontId="20" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment vertical="top"/>
     </xf>
-    <xf borderId="3" fillId="7" fontId="21" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="3" fillId="7" fontId="22" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment vertical="top"/>
     </xf>
-    <xf borderId="0" fillId="14" fontId="19" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+    <xf borderId="0" fillId="14" fontId="20" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment vertical="bottom"/>
     </xf>
-    <xf borderId="3" fillId="14" fontId="19" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="3" fillId="14" fontId="20" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment vertical="top"/>
     </xf>
-    <xf borderId="3" fillId="14" fontId="19" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="3" fillId="14" fontId="20" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
-    <xf borderId="3" fillId="14" fontId="22" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="3" fillId="14" fontId="23" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
-    </xf>
-    <xf borderId="3" fillId="14" fontId="23" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment vertical="top"/>
     </xf>
     <xf borderId="3" fillId="14" fontId="24" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment vertical="top"/>
     </xf>
+    <xf borderId="3" fillId="14" fontId="25" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment vertical="top"/>
+    </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="3" fillId="14" fontId="24" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="3" fillId="14" fontId="25" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2338,7 +2343,7 @@
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <x18tc:personList xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <x18tc:person displayName="Phil Reed" id="{36c4ad88-d8b2-42ad-96d4-b9483560a789}" providerId="google-sheets"/>
+  <x18tc:person displayName="Phil Reed" id="{a9323ab0-2d30-4248-86a4-acdccfd67e7e}" providerId="google-sheets"/>
 </x18tc:personList>
 </file>
 
@@ -2538,47 +2543,47 @@
 
 <file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
 <x18tc:ThreadedComments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:xltc2="http://schemas.microsoft.com/office/spreadsheetml/2020/threadedcomments2" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <x18tc:threadedComment ref="N42" dT="2026-06-10T08:21:58.00" personId="{36c4ad88-d8b2-42ad-96d4-b9483560a789}" id="{c93ec52d-3811-4e8e-8987-a0e04d67fed5}" done="0">
+  <x18tc:threadedComment ref="N42" dT="2026-06-10T08:21:58.00" personId="{a9323ab0-2d30-4248-86a4-acdccfd67e7e}" id="{b8c87507-4a8d-4067-bb0d-ad3535e9bfd0}" done="0">
     <x18tc:text xml:space="preserve">TODO: event types</x18tc:text>
   </x18tc:threadedComment>
-  <x18tc:threadedComment ref="N30" dT="2026-06-14T18:18:45.00" personId="{36c4ad88-d8b2-42ad-96d4-b9483560a789}" id="{efabe969-7dca-426e-acf9-b3c8261a837f}" done="1">
+  <x18tc:threadedComment ref="N30" dT="2026-06-14T18:18:45.00" personId="{a9323ab0-2d30-4248-86a4-acdccfd67e7e}" id="{34973966-2beb-456a-b13f-8d4c654fcc70}" done="1">
     <x18tc:text xml:space="preserve">Is this the best way to record timezone?</x18tc:text>
   </x18tc:threadedComment>
-  <x18tc:threadedComment ref="L1" dT="2026-04-16T07:15:59.00" personId="{36c4ad88-d8b2-42ad-96d4-b9483560a789}" id="{8fbcdf78-ef70-4737-aa2f-226525291599}" done="1">
+  <x18tc:threadedComment ref="L1" dT="2026-04-16T07:15:59.00" personId="{a9323ab0-2d30-4248-86a4-acdccfd67e7e}" id="{f52a97ab-1ac4-42b5-a810-0c62e3171378}" done="1">
     <x18tc:text xml:space="preserve">Still to define: controlled vocabularies</x18tc:text>
   </x18tc:threadedComment>
-  <x18tc:threadedComment ref="J16" dT="2026-04-16T07:35:15.00" personId="{36c4ad88-d8b2-42ad-96d4-b9483560a789}" id="{c2df04c0-8527-437b-935e-02e7db7acb5f}" done="0">
+  <x18tc:threadedComment ref="J16" dT="2026-04-16T07:35:15.00" personId="{a9323ab0-2d30-4248-86a4-acdccfd67e7e}" id="{419191be-88a2-4ebb-a9d0-45b001253b72}" done="0">
     <x18tc:text xml:space="preserve">EOSC 2024 schema has 'Expertise Level'. TeSS has 'Competency Level' and the Bioschemas 'educationalLevel' property, limited to the values of 'Beginner', 'Intermediate', 'Advanced'. 
 This might be better represented as two separate properties. Consider Terms4FAIRskills vocabulary for one of these.</x18tc:text>
   </x18tc:threadedComment>
-  <x18tc:threadedComment ref="L35" dT="2026-04-16T18:33:19.00" personId="{36c4ad88-d8b2-42ad-96d4-b9483560a789}" id="{797089d9-9fef-4104-a3bd-35403993da1d}" done="0">
+  <x18tc:threadedComment ref="L35" dT="2026-04-16T18:33:19.00" personId="{a9323ab0-2d30-4248-86a4-acdccfd67e7e}" id="{492be683-d186-43f6-8398-65826dbb9411}" done="0">
     <x18tc:text xml:space="preserve">Could use 2 or 3 character ISO 3166 country code</x18tc:text>
   </x18tc:threadedComment>
-  <x18tc:threadedComment ref="J47" dT="2026-04-16T07:36:05.00" personId="{36c4ad88-d8b2-42ad-96d4-b9483560a789}" id="{0c56af75-6606-4500-b0e0-efb6e4ee024c}" done="1">
+  <x18tc:threadedComment ref="J47" dT="2026-04-16T07:36:05.00" personId="{a9323ab0-2d30-4248-86a4-acdccfd67e7e}" id="{4e41cf75-544b-4e1e-a9ca-ddfa81e299ad}" done="1">
     <x18tc:text xml:space="preserve">Required if exists</x18tc:text>
   </x18tc:threadedComment>
-  <x18tc:threadedComment ref="N18" dT="2026-06-10T08:11:40.00" personId="{36c4ad88-d8b2-42ad-96d4-b9483560a789}" id="{711133ba-b785-4ddc-91ee-65c1a80128d2}" done="0">
+  <x18tc:threadedComment ref="N18" dT="2026-06-10T08:11:40.00" personId="{a9323ab0-2d30-4248-86a4-acdccfd67e7e}" id="{86067411-4f64-4dea-bb8c-484eb0624e97}" done="0">
     <x18tc:text xml:space="preserve">Add to Bioschemas</x18tc:text>
   </x18tc:threadedComment>
-  <x18tc:threadedComment ref="K32" dT="2026-04-16T07:35:24.00" personId="{36c4ad88-d8b2-42ad-96d4-b9483560a789}" id="{194dfa0d-f86e-48fa-aa6a-8fca58e121aa}" done="1">
+  <x18tc:threadedComment ref="K32" dT="2026-04-16T07:35:24.00" personId="{a9323ab0-2d30-4248-86a4-acdccfd67e7e}" id="{655fe435-7a29-4e9b-a1f1-627dbaa873fa}" done="1">
     <x18tc:text xml:space="preserve">Expand on this</x18tc:text>
   </x18tc:threadedComment>
-  <x18tc:threadedComment ref="L7" dT="2026-04-16T16:10:50.00" personId="{36c4ad88-d8b2-42ad-96d4-b9483560a789}" id="{e76141e3-8a70-4937-9879-b614dd0e3767}" done="1">
+  <x18tc:threadedComment ref="L7" dT="2026-04-16T16:10:50.00" personId="{a9323ab0-2d30-4248-86a4-acdccfd67e7e}" id="{5fbae45b-a0ee-4e46-816c-a61f09720000}" done="1">
     <x18tc:text xml:space="preserve">TeSS currently supports two "levels" of material contribution: 'author' and 'contributor'. For events, this changes to 'Organizer' which may be a person or an organization. Our workshop proposed extending this beyond author and contributor, to an existing CV. It is not clear to me from the notes which is suitable. (We also propose including ORCID for 'organizer' of an event'.)</x18tc:text>
   </x18tc:threadedComment>
-  <x18tc:threadedComment ref="J12" dT="2026-04-16T18:21:29.00" personId="{36c4ad88-d8b2-42ad-96d4-b9483560a789}" id="{eb3bd140-efca-406a-8d17-195ddc05469c}" done="0">
+  <x18tc:threadedComment ref="J12" dT="2026-04-16T18:21:29.00" personId="{a9323ab0-2d30-4248-86a4-acdccfd67e7e}" id="{5958f09c-2156-4518-8c68-755ee955ef16}" done="0">
     <x18tc:text xml:space="preserve">Base TeSS does not mandate license, too many materials would be rejected. 
 Also, TeSS events do not have license (it is not in the Bioschemas profile).</x18tc:text>
   </x18tc:threadedComment>
-  <x18tc:threadedComment ref="N7" dT="2026-06-10T07:53:50.00" personId="{36c4ad88-d8b2-42ad-96d4-b9483560a789}" id="{799f37c3-35ee-48b3-8d2f-783c9ecca11b}" done="0">
+  <x18tc:threadedComment ref="N7" dT="2026-06-10T07:53:50.00" personId="{a9323ab0-2d30-4248-86a4-acdccfd67e7e}" id="{7513edb4-21ae-4d7f-a667-8b566e125b23}" done="0">
     <x18tc:text xml:space="preserve">TODO: Role</x18tc:text>
   </x18tc:threadedComment>
-  <x18tc:threadedComment ref="J7" dT="2026-04-16T18:39:59.00" personId="{36c4ad88-d8b2-42ad-96d4-b9483560a789}" id="{14a075e4-3e63-45dd-873b-d4b67be1f443}" done="0">
+  <x18tc:threadedComment ref="J7" dT="2026-04-16T18:39:59.00" personId="{a9323ab0-2d30-4248-86a4-acdccfd67e7e}" id="{4f1e0add-0afa-4f26-a2f2-76800d1c42cc}" done="0">
     <x18tc:text xml:space="preserve">TeSS currently supports two "levels" of material contribution: 'author' and 'contributor'. For events, this changes to 'Organizer' which may be a person or an organization. 
 Our workshop proposed extending this beyond author and contributor, to an existing CV. It is not clear to me from the notes which is suitable. 
 (We also propose including ORCID for 'organizer' of an event'.)</x18tc:text>
   </x18tc:threadedComment>
-  <x18tc:threadedComment ref="L42" dT="2026-04-16T18:38:01.00" personId="{36c4ad88-d8b2-42ad-96d4-b9483560a789}" id="{1ce51903-2067-4d3a-ac25-0103b7cbba14}" done="0">
+  <x18tc:threadedComment ref="L42" dT="2026-04-16T18:38:01.00" personId="{a9323ab0-2d30-4248-86a4-acdccfd67e7e}" id="{9b74a778-7338-4d64-b624-90b4eaee3552}" done="0">
     <x18tc:text xml:space="preserve">Event type vocabulary TBD.
 How TeSS ingests event type now: If the text "online" appears in the value, event will be set to "Online" in TeSS, otherwise "Face-to-face". Hybrid is currently not supported [DReSA creates two events for this.]. Will also be set to "Online" if "location" is using the type "VirtualLocation"</x18tc:text>
   </x18tc:threadedComment>
@@ -10558,13 +10563,14 @@
     <hyperlink r:id="rId7" ref="N12"/>
     <hyperlink r:id="rId8" ref="N13"/>
     <hyperlink r:id="rId9" ref="N19"/>
-    <hyperlink r:id="rId10" ref="U34"/>
-    <hyperlink r:id="rId11" ref="U35"/>
-    <hyperlink r:id="rId12" location=".YrHnEi8iu-o" ref="N42"/>
-    <hyperlink r:id="rId13" ref="N47"/>
+    <hyperlink r:id="rId10" ref="N30"/>
+    <hyperlink r:id="rId11" ref="U34"/>
+    <hyperlink r:id="rId12" ref="U35"/>
+    <hyperlink r:id="rId13" location=".YrHnEi8iu-o" ref="N42"/>
+    <hyperlink r:id="rId14" ref="N47"/>
   </hyperlinks>
-  <drawing r:id="rId14"/>
-  <legacyDrawing r:id="rId15"/>
+  <drawing r:id="rId15"/>
+  <legacyDrawing r:id="rId16"/>
 </worksheet>
 </file>
 

</xml_diff>